<commit_message>
Bring the economy model (.xlsx) text in line with the corrected framing
Update the workbook's descriptive cells (README, Loan Desk, KPI Impact tabs)
so the model matches the case study after the HR review:

- Loan Desk relabelled a liquidity lock with a hard-currency sink; the soft
  side is described as a faucet by design.
- Guardrail #6 corrected — it no longer claims the Desk "drains cash on net";
  the net drain is the hard-currency ingot sink, with the boost cap as the
  anti-inflation control.
- Resequenced-interstitial note now names it as the main retention risk behind
  a D1/session-length guardrail.
- A/B design wording: sweep the tuning curve rather than "on/off".

Edited shared-string text only; charts, styles, and the 400+ formulas are
byte-for-byte unchanged. Validated: zip integrity OK, all XML well-formed,
string counts preserved.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DuTW2YjwUTpjHacJYHnGy
</commit_message>
<xml_diff>
--- a/Idle_Bank_Tycoon_Economy_Model.xlsx
+++ b/Idle_Bank_Tycoon_Economy_Model.xlsx
@@ -31,7 +31,7 @@
     <t xml:space="preserve">IDLE BANK TYCOON  ·  GAME ECONOMY CASE STUDY</t>
   </si>
   <si>
-    <t xml:space="preserve">A working economy model: (A) a soft-currency sink feature  +  (B) rewarded-ad reward tuning</t>
+    <t xml:space="preserve">A working economy model: (A) a liquidity-lock engagement mechanic (hard-currency sink)  +  (B) rewarded-ad reward tuning</t>
   </si>
   <si>
     <t xml:space="preserve">PURPOSE</t>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">3.</t>
   </si>
   <si>
-    <t xml:space="preserve">Loan Desk (Option A) models a soft-currency sink that converts idle cash into a temporary income multiplier.</t>
+    <t xml:space="preserve">Loan Desk (Option A) models a liquidity-lock mechanic that converts idle cash into a temporary income multiplier. On soft currency it is a faucet by design; its true currency sink is hard-currency (ingots).</t>
   </si>
   <si>
     <t xml:space="preserve">4.</t>
@@ -388,16 +388,16 @@
     <t xml:space="preserve">"Cost growth (1.21x) outpaces income growth (1.18x), yet the 12h offline cap lets cash pile up between the few upgrades that matter, and there is no compelling SINK to absorb it. That idle surplus is unused economic value and a missed monetisation touchpoint."</t>
   </si>
   <si>
-    <t xml:space="preserve">OPTION A  ·  THE LOAN DESK  (soft-currency sink)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Converts idle cash into a temporary income multiplier. Adds a real sink, a hard-currency touchpoint, and an active decision to the idle loop.</t>
+    <t xml:space="preserve">OPTION A  ·  THE LOAN DESK  (liquidity lock + hard-currency sink)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Converts idle cash into a temporary income multiplier. Adds a liquidity lock, a hard-currency touchpoint (the real currency sink), and an active decision to the idle loop.</t>
   </si>
   <si>
     <t xml:space="preserve">Concept</t>
   </si>
   <si>
-    <t xml:space="preserve">Players lock a share of their idle cash into a fixed-term 'loan'. While the loan runs, income/sec is boosted (the player is 'earning interest'). At maturity the principal returns plus a small soft bonus. Players may pay GOLD INGOTS to end a loan early (hard-currency sink) or to unlock extra loan slots. This drains the surplus the Baseline tab exposed, creates a meaningful choice (how much to lock, how long), and opens a non-ad monetisation lever, without pay-to-win, since rewards are time-based, not power-based.</t>
+    <t xml:space="preserve">Players lock a share of their idle cash into a fixed-term 'loan'. While the loan runs, income/sec is boosted (the player is 'earning interest'). At maturity the full principal returns plus a small bonus, so on soft currency the feature is a faucet by design, not a sink. Players may pay GOLD INGOTS to end a loan early (hard-currency sink) or to unlock extra loan slots. This removes liquidity from the surplus the Baseline tab exposed, creates a meaningful choice (how much to lock, how long), and opens a non-ad monetisation lever, without pay-to-win, since rewards are time-based, not power-based.</t>
   </si>
   <si>
     <t xml:space="preserve">Worked example: representative mid-game player</t>
@@ -526,7 +526,7 @@
     <t xml:space="preserve">Loan slots are limited (Parameters C37) so the feature can't dominate the session; extra slots are a paid sink.</t>
   </si>
   <si>
-    <t xml:space="preserve">Soft interest (Parameters C35) kept low so the Loan Desk drains cash on net rather than printing it.</t>
+    <t xml:space="preserve">Soft interest (Parameters C35) kept low and the boost capped, so soft inflation stays the cost curve's job (1.21x/lvl); the net currency drain is the hard-currency ingot sink, not the soft side.</t>
   </si>
   <si>
     <t xml:space="preserve">OPTION B  ·  REWARDED-AD REWARD TUNING</t>
@@ -625,7 +625,7 @@
     <t xml:space="preserve">Placement principle (free uplift, no extra ads)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sequence matters as much as frequency: industry tests show showing an interstitial AFTER a rewarded-video offer lifts ad ARPDAU ~+23% with no added frustration. Recommendation: keep rewarded ads opt-in and value-scaled (above), and A/B test interstitial sequencing at natural breakpoints (post-prestige, post-loan-maturity) rather than raising raw ad frequency.</t>
+    <t xml:space="preserve">Sequence matters as much as frequency: industry tests show showing an interstitial AFTER a rewarded-video offer lifts ad ARPDAU ~+23%. It also adds an impression at a sensitive moment, so it is the main retention risk here and ships only behind a D1/session-length guardrail. Recommendation: keep rewarded ads opt-in and value-scaled (above), and A/B test interstitial sequencing at natural breakpoints (post-prestige, post-loan-maturity) rather than raising raw ad frequency.</t>
   </si>
   <si>
     <t xml:space="preserve">KPI IMPACT  ·  COMBINED LEVERS &amp; SENSITIVITY</t>
@@ -694,7 +694,7 @@
     <t xml:space="preserve">Hypothesis A (Loan Desk)</t>
   </si>
   <si>
-    <t xml:space="preserve">Adding a soft-currency sink lifts D7 retention (more to do late-game) and ARPDAU (ingot sink) without hurting D1.</t>
+    <t xml:space="preserve">Adding the Loan Desk lifts D7 retention (more to do late-game) and ARPDAU (ingot sink) without hurting D1.</t>
   </si>
   <si>
     <t xml:space="preserve">Hypothesis B (Ad tuning)</t>
@@ -706,7 +706,7 @@
     <t xml:space="preserve">Design</t>
   </si>
   <si>
-    <t xml:space="preserve">Assign at install (new players only). Split by platform (iOS vs Android behave differently). 4–5 variants of reward size / loan multiplier, not just on/off.</t>
+    <t xml:space="preserve">Assign at install (new players only). Split by platform (iOS vs Android behave differently). 4–5 variants of reward size / loan multiplier, sweeping the range to find the tuning curve.</t>
   </si>
   <si>
     <t xml:space="preserve">Primary KPIs</t>
@@ -838,7 +838,7 @@
     <t xml:space="preserve">Tuned so yield stays below active-upgrade returns (anti-cannibalisation). A/B test the real values.</t>
   </si>
   <si>
-    <t xml:space="preserve">Loan adoption 45%; 8% of users buy a sink</t>
+    <t xml:space="preserve">Loan adoption 45%; 8% of users are ingot spenders</t>
   </si>
   <si>
     <t xml:space="preserve">Mid-range engagement-feature assumptions; validate live.</t>

</xml_diff>